<commit_message>
9/3 finished preliminary nutrient probe data analysis.
</commit_message>
<xml_diff>
--- a/Legacy effect/raw-data/VFT fire history/excel fire histories.xlsx
+++ b/Legacy effect/raw-data/VFT fire history/excel fire histories.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\VFT\VFT_github\zyao78VFTcode\raw-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390E4BC5-11BC-4AEC-9D11-DD2D15966486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EABE9DD0-1223-4EC3-BCDC-7AB09204338E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="3" xr2:uid="{58B67793-E89C-414F-A104-ABAD252BA177}"/>
+    <workbookView xWindow="45960" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{58B67793-E89C-414F-A104-ABAD252BA177}"/>
   </bookViews>
   <sheets>
     <sheet name="manager" sheetId="1" r:id="rId1"/>
     <sheet name="field_notes" sheetId="2" r:id="rId2"/>
     <sheet name="landsat" sheetId="3" r:id="rId3"/>
-    <sheet name="landscape" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">field_notes!$A$1:$G$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">manager!$A$2:$E$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">manager!$A$2:$E$62</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="65">
   <si>
     <t>FILE CURRENT AS OF 2/24/25</t>
   </si>
@@ -197,6 +196,10 @@
     <t>fire in 2018-03-01 did not reach our plots</t>
   </si>
   <si>
+    <t>FILE CURRENT AS OF 8/27/25</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
     <t>GSP-BI</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
@@ -238,35 +241,15 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>FILE CURRENT AS OF 11/14/25</t>
+    <t>FILE CURRENT AS OF 9/1/26</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>FILE CURRENT AS OF 11/14/25</t>
+    <t>VFT&gt;VFT fire history data&gt;Email records&gt;GSP_ZacharyWest_2025_2026.pdf</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve"> landscape fire records were produced based on the manager records. Occurrences of fires were confirmed using Landsat false color images (SWIR, NIR, Blue).</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>startyear</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>CH</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>CM</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>IA</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>ME</t>
+    <t>N</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -274,7 +257,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -316,6 +299,12 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -343,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -356,6 +345,7 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -743,19 +733,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B609A7-77BB-AE4A-B6B2-C4ACEA0133DD}">
-  <dimension ref="A1:G61"/>
-  <sheetFormatPr defaultColWidth="10.87890625" defaultRowHeight="15" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G63"/>
+  <sheetFormatPr defaultColWidth="10.87890625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="4" max="4" width="82.87890625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="34.9" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="34.9">
       <c r="A1" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -778,7 +768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7">
       <c r="A3" s="7">
         <v>39508</v>
       </c>
@@ -796,7 +786,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7">
       <c r="A4" s="7">
         <v>41343</v>
       </c>
@@ -814,7 +804,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7">
       <c r="A5" s="7">
         <v>42529</v>
       </c>
@@ -834,7 +824,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7">
       <c r="A6" s="7">
         <v>43540</v>
       </c>
@@ -852,7 +842,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7">
       <c r="A7" s="7">
         <v>44707</v>
       </c>
@@ -870,7 +860,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7">
       <c r="A8" s="7">
         <v>45777</v>
       </c>
@@ -886,7 +876,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7">
       <c r="A9" s="7">
         <v>39600</v>
       </c>
@@ -904,7 +894,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7">
       <c r="A10" s="7">
         <v>42532</v>
       </c>
@@ -924,7 +914,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7">
       <c r="A11" s="7">
         <v>43540</v>
       </c>
@@ -942,7 +932,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7">
       <c r="A12" s="7">
         <v>44707</v>
       </c>
@@ -960,7 +950,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7">
       <c r="A13" s="8">
         <v>33664</v>
       </c>
@@ -978,7 +968,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7">
       <c r="A14" s="8">
         <v>34363</v>
       </c>
@@ -996,7 +986,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7">
       <c r="A15" s="8">
         <v>34747</v>
       </c>
@@ -1014,7 +1004,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7">
       <c r="A16" s="8">
         <v>35087</v>
       </c>
@@ -1032,7 +1022,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6">
       <c r="A17" s="8">
         <v>35525</v>
       </c>
@@ -1050,7 +1040,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6">
       <c r="A18" s="8">
         <v>36242</v>
       </c>
@@ -1068,7 +1058,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6">
       <c r="A19" s="8">
         <v>36917</v>
       </c>
@@ -1086,7 +1076,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6">
       <c r="A20" s="8">
         <v>37690</v>
       </c>
@@ -1104,7 +1094,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6">
       <c r="A21" s="8">
         <v>38389</v>
       </c>
@@ -1122,7 +1112,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6">
       <c r="A22" s="8">
         <v>40567</v>
       </c>
@@ -1140,7 +1130,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6">
       <c r="A23" s="8">
         <v>40942</v>
       </c>
@@ -1158,7 +1148,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6">
       <c r="A24" s="8">
         <v>41315</v>
       </c>
@@ -1176,7 +1166,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6">
       <c r="A25" s="8">
         <v>42202</v>
       </c>
@@ -1194,7 +1184,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6">
       <c r="A26" s="8">
         <v>42817</v>
       </c>
@@ -1212,7 +1202,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6">
       <c r="A27" s="8">
         <v>44235</v>
       </c>
@@ -1230,7 +1220,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6">
       <c r="A28" s="8">
         <v>45068</v>
       </c>
@@ -1248,27 +1238,27 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A29" s="7">
+    <row r="29" spans="1:6">
+      <c r="A29" s="10">
+        <v>45749</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" s="5"/>
+      <c r="F29" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="7">
         <v>38381</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A30" s="7">
-        <v>39027</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>22</v>
@@ -1284,9 +1274,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6">
       <c r="A31" s="7">
-        <v>40134</v>
+        <v>39027</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>22</v>
@@ -1302,12 +1292,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6">
       <c r="A32" s="7">
-        <v>38737</v>
+        <v>40134</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>9</v>
@@ -1315,19 +1305,14 @@
       <c r="D32" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="E32" s="5"/>
       <c r="F32" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" s="7">
-        <v>39094</v>
+        <v>38737</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>24</v>
@@ -1348,9 +1333,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7">
       <c r="A34" s="7">
-        <v>39850</v>
+        <v>39094</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>24</v>
@@ -1371,9 +1356,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7">
       <c r="A35" s="7">
-        <v>40015</v>
+        <v>39850</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>24</v>
@@ -1384,14 +1369,19 @@
       <c r="D35" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E35" s="5"/>
+      <c r="E35" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="F35" s="5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="G35" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" s="7">
-        <v>40978</v>
+        <v>40015</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>24</v>
@@ -1402,17 +1392,14 @@
       <c r="D36" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E36" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="E36" s="5"/>
       <c r="F36" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G36" s="5"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.4">
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="7">
-        <v>40980</v>
+        <v>40978</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>24</v>
@@ -1429,13 +1416,11 @@
       <c r="F37" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G37" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="G37" s="5"/>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" s="7">
-        <v>42430</v>
+        <v>40980</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>24</v>
@@ -1444,16 +1429,21 @@
         <v>9</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E38" s="5"/>
+        <v>23</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="F38" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
+        <v>13</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="7">
-        <v>42915</v>
+        <v>42430</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>24</v>
@@ -1462,21 +1452,16 @@
         <v>9</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>25</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="E39" s="5"/>
       <c r="F39" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" s="7">
-        <v>43156</v>
+        <v>42915</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>24</v>
@@ -1487,14 +1472,19 @@
       <c r="D40" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E40" s="5"/>
+      <c r="E40" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="F40" s="5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="G40" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" s="7">
-        <v>43892</v>
+        <v>43156</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>24</v>
@@ -1503,16 +1493,16 @@
         <v>9</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E41" s="5"/>
       <c r="F41" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7">
       <c r="A42" s="7">
-        <v>44624</v>
+        <v>43892</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>24</v>
@@ -1521,34 +1511,34 @@
         <v>9</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E42" s="5"/>
       <c r="F42" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7">
       <c r="A43" s="7">
-        <v>40939</v>
+        <v>44624</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E43" s="5"/>
       <c r="F43" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7">
       <c r="A44" s="7">
-        <v>42048</v>
+        <v>40939</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>29</v>
@@ -1564,9 +1554,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7">
       <c r="A45" s="7">
-        <v>43871</v>
+        <v>42048</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>29</v>
@@ -1574,35 +1564,35 @@
       <c r="C45" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D45" s="5" t="s">
-        <v>31</v>
+      <c r="D45" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7">
       <c r="A46" s="7">
-        <v>32904</v>
+        <v>43871</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7">
       <c r="A47" s="7">
-        <v>34001</v>
+        <v>32904</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>32</v>
@@ -1618,9 +1608,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7">
       <c r="A48" s="7">
-        <v>34747</v>
+        <v>34001</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>32</v>
@@ -1636,9 +1626,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6">
       <c r="A49" s="7">
-        <v>35845</v>
+        <v>34747</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>32</v>
@@ -1654,9 +1644,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6">
       <c r="A50" s="7">
-        <v>37663</v>
+        <v>35845</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>32</v>
@@ -1672,9 +1662,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6">
       <c r="A51" s="7">
-        <v>39083</v>
+        <v>37663</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>32</v>
@@ -1690,9 +1680,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6">
       <c r="A52" s="7">
-        <v>40205</v>
+        <v>39083</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>32</v>
@@ -1708,9 +1698,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6">
       <c r="A53" s="7">
-        <v>41294</v>
+        <v>40205</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>32</v>
@@ -1726,9 +1716,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6">
       <c r="A54" s="7">
-        <v>42024</v>
+        <v>41294</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>32</v>
@@ -1744,9 +1734,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6">
       <c r="A55" s="7">
-        <v>42962</v>
+        <v>42024</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>32</v>
@@ -1762,9 +1752,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6">
       <c r="A56" s="7">
-        <v>43696</v>
+        <v>42962</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>32</v>
@@ -1780,9 +1770,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6">
       <c r="A57" s="7">
-        <v>44970</v>
+        <v>43696</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>32</v>
@@ -1798,45 +1788,45 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6">
       <c r="A58" s="7">
-        <v>40939</v>
+        <v>44970</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D58" s="9" t="s">
-        <v>30</v>
+      <c r="D58" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A59" s="7">
-        <v>42048</v>
+    <row r="59" spans="1:6">
+      <c r="A59" s="10">
+        <v>46091</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D59" s="9" t="s">
-        <v>30</v>
+      <c r="D59" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="E59" s="5"/>
-      <c r="F59" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F59" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
       <c r="A60" s="7">
-        <v>43900</v>
+        <v>40939</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>33</v>
@@ -1844,24 +1834,60 @@
       <c r="C60" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D60" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="7">
+        <v>42048</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="7">
+        <v>43900</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E60" s="5" t="s">
+      <c r="E62" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F60" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="D61" s="3"/>
+      <c r="F62" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="D63" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:E60" xr:uid="{E7B609A7-77BB-AE4A-B6B2-C4ACEA0133DD}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:E60">
-    <sortCondition ref="B3:B60"/>
-    <sortCondition ref="A3:A60"/>
+  <autoFilter ref="A2:E62" xr:uid="{E7B609A7-77BB-AE4A-B6B2-C4ACEA0133DD}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:E62">
+    <sortCondition ref="B3:B62"/>
+    <sortCondition ref="A3:A62"/>
   </sortState>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1872,14 +1898,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C5F246-917A-DB45-9A6A-503E61453CAC}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="10.87890625" defaultRowHeight="15" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="10.87890625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="34.9" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="34.9">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" s="5" customFormat="1">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -1902,7 +1928,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" s="5" customFormat="1">
       <c r="A3" s="7">
         <v>43540</v>
       </c>
@@ -1925,7 +1951,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" s="5" customFormat="1">
       <c r="A4" s="7">
         <v>44707</v>
       </c>
@@ -1948,7 +1974,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" s="5" customFormat="1">
       <c r="A5" s="7">
         <v>42532</v>
       </c>
@@ -1971,7 +1997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" s="5" customFormat="1">
       <c r="A6" s="7">
         <v>44707</v>
       </c>
@@ -1994,7 +2020,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" s="5" customFormat="1">
       <c r="A7" s="8">
         <v>45068</v>
       </c>
@@ -2017,7 +2043,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" s="5" customFormat="1">
       <c r="A8" s="7">
         <v>42430</v>
       </c>
@@ -2037,7 +2063,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" s="5" customFormat="1">
       <c r="A9" s="7">
         <v>43156</v>
       </c>
@@ -2060,7 +2086,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" s="5" customFormat="1">
       <c r="A10" s="7">
         <v>43892</v>
       </c>
@@ -2083,7 +2109,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" s="5" customFormat="1">
       <c r="A11" s="7">
         <v>44624</v>
       </c>
@@ -2106,7 +2132,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" s="5" customFormat="1">
       <c r="A12" s="7">
         <v>43871</v>
       </c>
@@ -2129,7 +2155,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" s="5" customFormat="1">
       <c r="A13" s="7">
         <v>43696</v>
       </c>
@@ -2152,7 +2178,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" s="5" customFormat="1">
       <c r="A14" s="7">
         <v>43900</v>
       </c>
@@ -2175,7 +2201,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" s="5" customFormat="1">
       <c r="A15" s="7">
         <v>44256</v>
       </c>
@@ -2195,7 +2221,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" s="5" customFormat="1">
       <c r="A16" s="7">
         <v>42795</v>
       </c>
@@ -2218,7 +2244,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" s="5" customFormat="1">
       <c r="A17" s="7">
         <v>44256</v>
       </c>
@@ -2238,7 +2264,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" s="5" customFormat="1">
       <c r="A18" s="7">
         <v>42795</v>
       </c>
@@ -2261,7 +2287,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" s="5" customFormat="1">
       <c r="A19" s="7">
         <v>44986</v>
       </c>
@@ -2281,7 +2307,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" s="5" customFormat="1">
       <c r="A20" s="7">
         <v>42795</v>
       </c>
@@ -2310,15 +2336,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31D715BE-6D22-334F-97CD-3B59221D3F48}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultColWidth="10.87890625" defaultRowHeight="15" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G36"/>
+  <sheetFormatPr defaultColWidth="10.87890625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="34.9" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="34.9">
       <c r="A1" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2341,221 +2367,221 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7">
       <c r="A3" s="1">
         <v>38443</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="1">
+        <v>39265</v>
+      </c>
+      <c r="B4" t="s">
         <v>51</v>
       </c>
-      <c r="D3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A4" s="1">
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="1">
         <v>40593</v>
       </c>
-      <c r="B4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
         <v>51</v>
       </c>
-      <c r="D4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A5" s="1">
+      <c r="C5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="1">
         <v>41363</v>
       </c>
-      <c r="B5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>51</v>
       </c>
-      <c r="D5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A6" s="1">
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="1">
         <v>42818</v>
       </c>
-      <c r="B6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
         <v>51</v>
       </c>
-      <c r="D6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A7" s="1">
+      <c r="C7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="1">
         <v>39123</v>
       </c>
-      <c r="B7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A8" s="1">
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="1">
         <v>40213</v>
       </c>
-      <c r="B8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A9" s="1">
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="1">
         <v>41363</v>
       </c>
-      <c r="B9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A10" s="1">
+      <c r="B10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="1">
         <v>42017</v>
       </c>
-      <c r="B10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A11" s="1">
+      <c r="B11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="1">
         <v>43690</v>
       </c>
-      <c r="B11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A12" s="1">
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="1">
         <v>44993</v>
-      </c>
-      <c r="B12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A13" s="1">
-        <v>38768</v>
       </c>
       <c r="B13" t="s">
         <v>55</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F13" t="s">
         <v>11</v>
@@ -2564,98 +2590,98 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7">
       <c r="A14" s="1">
+        <v>38768</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="1">
         <v>39857</v>
       </c>
-      <c r="B14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" t="s">
-        <v>52</v>
-      </c>
-      <c r="F14" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A15" s="1">
+      <c r="B15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="1">
         <v>42046</v>
       </c>
-      <c r="B15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A16" s="1">
+      <c r="B16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="1">
         <v>43870</v>
       </c>
-      <c r="B16" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A17" s="1">
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="1">
         <v>45054</v>
-      </c>
-      <c r="B17" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A18" s="1">
-        <v>36842</v>
       </c>
       <c r="B18" t="s">
         <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F18" t="s">
         <v>11</v>
@@ -2664,58 +2690,58 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7">
       <c r="A19" s="1">
+        <v>36842</v>
+      </c>
+      <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="1">
         <v>38388</v>
       </c>
-      <c r="B19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A20" s="1">
+      <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="1">
         <v>44286</v>
-      </c>
-      <c r="B20" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A21" s="1">
-        <v>35359</v>
       </c>
       <c r="B21" t="s">
         <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F21" t="s">
         <v>11</v>
@@ -2724,98 +2750,98 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7">
       <c r="A22" s="1">
+        <v>35359</v>
+      </c>
+      <c r="B22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="1">
         <v>36554</v>
       </c>
-      <c r="B22" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" t="s">
-        <v>52</v>
-      </c>
-      <c r="F22" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A23" s="1">
+      <c r="B23" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="1">
         <v>42462</v>
       </c>
-      <c r="B23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" t="s">
-        <v>52</v>
-      </c>
-      <c r="F23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A24" s="1">
+      <c r="B24" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="1">
         <v>43902</v>
       </c>
-      <c r="B24" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" t="s">
-        <v>51</v>
-      </c>
-      <c r="D24" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A25" s="1">
+      <c r="B25" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="1">
         <v>44654</v>
-      </c>
-      <c r="B25" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" t="s">
-        <v>52</v>
-      </c>
-      <c r="F25" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A26" s="1">
-        <v>38362</v>
       </c>
       <c r="B26" t="s">
         <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D26" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F26" t="s">
         <v>11</v>
@@ -2824,18 +2850,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7">
       <c r="A27" s="1">
-        <v>39971</v>
+        <v>38362</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F27" t="s">
         <v>11</v>
@@ -2844,58 +2870,58 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7">
       <c r="A28" s="1">
+        <v>39983</v>
+      </c>
+      <c r="B28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D28" t="s">
+        <v>53</v>
+      </c>
+      <c r="F28" t="s">
+        <v>11</v>
+      </c>
+      <c r="G28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="1">
+        <v>40334</v>
+      </c>
+      <c r="B29" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" t="s">
+        <v>53</v>
+      </c>
+      <c r="F29" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="1">
         <v>42783</v>
-      </c>
-      <c r="B28" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28" t="s">
-        <v>51</v>
-      </c>
-      <c r="D28" t="s">
-        <v>52</v>
-      </c>
-      <c r="F28" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A29" s="1">
-        <v>43902</v>
-      </c>
-      <c r="B29" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" t="s">
-        <v>51</v>
-      </c>
-      <c r="D29" t="s">
-        <v>52</v>
-      </c>
-      <c r="F29" t="s">
-        <v>11</v>
-      </c>
-      <c r="G29" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A30" s="1">
-        <v>39560</v>
       </c>
       <c r="B30" t="s">
         <v>59</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F30" t="s">
         <v>11</v>
@@ -2904,467 +2930,124 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7">
       <c r="A31" s="1">
+        <v>43902</v>
+      </c>
+      <c r="B31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" t="s">
+        <v>53</v>
+      </c>
+      <c r="F31" t="s">
+        <v>11</v>
+      </c>
+      <c r="G31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="1">
+        <v>44735</v>
+      </c>
+      <c r="B32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" t="s">
+        <v>53</v>
+      </c>
+      <c r="F32" t="s">
+        <v>11</v>
+      </c>
+      <c r="G32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="1">
+        <v>39560</v>
+      </c>
+      <c r="B33" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+      <c r="F33" t="s">
+        <v>11</v>
+      </c>
+      <c r="G33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="1">
         <v>34777</v>
       </c>
-      <c r="B31" t="s">
-        <v>60</v>
-      </c>
-      <c r="C31" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" t="s">
-        <v>52</v>
-      </c>
-      <c r="F31" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A32" s="1">
+      <c r="B34" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" t="s">
+        <v>53</v>
+      </c>
+      <c r="F34" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="1">
         <v>31433</v>
       </c>
-      <c r="B32" t="s">
-        <v>60</v>
-      </c>
-      <c r="C32" t="s">
-        <v>51</v>
-      </c>
-      <c r="D32" t="s">
-        <v>52</v>
-      </c>
-      <c r="F32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G32" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A33" s="1">
+      <c r="B35" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" t="s">
+        <v>53</v>
+      </c>
+      <c r="F35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="1">
         <v>31929</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B36" t="s">
         <v>17</v>
       </c>
-      <c r="C33" t="s">
-        <v>51</v>
-      </c>
-      <c r="D33" t="s">
-        <v>52</v>
-      </c>
-      <c r="F33" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E1E58FE-7144-4B59-9820-C76451FCA0F7}">
-  <dimension ref="A1:H48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.4"/>
-  <sheetData>
-    <row r="1" spans="1:8" ht="34.9" x14ac:dyDescent="0.9">
-      <c r="A1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3">
-        <v>2007</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4">
-        <v>2012</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A5">
-        <v>2015</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A6">
-        <v>2018</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A7">
-        <v>2021</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8">
-        <v>2024</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A9">
-        <v>1994</v>
-      </c>
-      <c r="B9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A10">
-        <v>2007</v>
-      </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A11">
-        <v>2015</v>
-      </c>
-      <c r="B11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A12">
-        <v>2018</v>
-      </c>
-      <c r="B12" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A13">
-        <v>2021</v>
-      </c>
-      <c r="B13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A14">
-        <v>2004</v>
-      </c>
-      <c r="B14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A15">
-        <v>2010</v>
-      </c>
-      <c r="B15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A16">
-        <v>2011</v>
-      </c>
-      <c r="B16" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A17">
-        <v>2012</v>
-      </c>
-      <c r="B17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A18">
-        <v>2015</v>
-      </c>
-      <c r="B18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A19">
-        <v>2016</v>
-      </c>
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A20">
-        <v>2020</v>
-      </c>
-      <c r="B20" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A21">
-        <v>2022</v>
-      </c>
-      <c r="B21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A22">
-        <v>2002</v>
-      </c>
-      <c r="B22" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A23">
-        <v>2006</v>
-      </c>
-      <c r="B23" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A24">
-        <v>2009</v>
-      </c>
-      <c r="B24" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A25">
-        <v>2012</v>
-      </c>
-      <c r="B25" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A26">
-        <v>2014</v>
-      </c>
-      <c r="B26" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A27">
-        <v>2017</v>
-      </c>
-      <c r="B27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A28">
-        <v>2019</v>
-      </c>
-      <c r="B28" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A29">
-        <v>2022</v>
-      </c>
-      <c r="B29" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A30">
-        <v>2004</v>
-      </c>
-      <c r="B30" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A31">
-        <v>2006</v>
-      </c>
-      <c r="B31" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A32">
-        <v>2009</v>
-      </c>
-      <c r="B32" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A33">
-        <v>2020</v>
-      </c>
-      <c r="B33" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A34">
-        <v>2005</v>
-      </c>
-      <c r="B34" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A35">
-        <v>2008</v>
-      </c>
-      <c r="B35" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A36">
-        <v>2011</v>
-      </c>
-      <c r="B36" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A37">
-        <v>2015</v>
-      </c>
-      <c r="B37" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A38">
-        <v>2017</v>
-      </c>
-      <c r="B38" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A39">
-        <v>2019</v>
-      </c>
-      <c r="B39" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A40">
-        <v>2021</v>
-      </c>
-      <c r="B40" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A41">
-        <v>2011</v>
-      </c>
-      <c r="B41" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A42">
-        <v>2014</v>
-      </c>
-      <c r="B42" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A43">
-        <v>2019</v>
-      </c>
-      <c r="B43" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A44">
-        <v>2022</v>
-      </c>
-      <c r="B44" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A45">
-        <v>2004</v>
-      </c>
-      <c r="B45" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A46">
-        <v>2008</v>
-      </c>
-      <c r="B46" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A47">
-        <v>2016</v>
-      </c>
-      <c r="B47" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A48">
-        <v>2019</v>
-      </c>
-      <c r="B48" t="s">
-        <v>68</v>
+      <c r="C36" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" t="s">
+        <v>53</v>
+      </c>
+      <c r="F36" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>